<commit_message>
all updates (replaced videos, added kiosk view, cue review/control, credits, etc)
</commit_message>
<xml_diff>
--- a/CTC_Backend/chat_log.xlsx
+++ b/CTC_Backend/chat_log.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C27"/>
+  <dimension ref="A1:C26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="14.6640625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -845,34 +845,17 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-08-31 16:43:37</t>
+          <t>2026-09-04 18:45:15</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>A black liberated reality has no fear and allows for joy and freedom</t>
+          <t>freedom please</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>What does this liberation mean to you? How does it manifest in your daily life, and what kind of freedom would you like to experience in this reality?</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>2026-08-31 16:44:23</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>No pain, no more Black people being lynched</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>What would it take to create a world where the pain and suffering of the past can be acknowledged and healed, rather than perpetuated? How can we work towards a future where Black people are truly safe and valued?</t>
+          <t>What does freedom mean to you, in this moment? Is it the ability to break free from constraints, or to find liberation from within?</t>
         </is>
       </c>
     </row>

</xml_diff>